<commit_message>
S10: anexos A-F de Alto Selva (modelo, vistas, estructura de la informacion, brechas con formulas y seccion 5 en PDF)
</commit_message>
<xml_diff>
--- a/docs/evidencias/S10/anexo_C_estructura_informacion.xlsx
+++ b/docs/evidencias/S10/anexo_C_estructura_informacion.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -490,7 +490,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>DICOSUR · PETI v0.10 · Restringido · Taller 10 SI-886</t>
+          <t>Municipalidad Distrital de Alto Selva · PETI v0.10 · Restringido · Taller 10 SI-886</t>
         </is>
       </c>
     </row>
@@ -549,22 +549,22 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Cliente</t>
+          <t>Contribuyente y predio</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>ERP; Portal B2B; Hoja comercial</t>
+          <t>Rentas y catastro; Caja; Mesa de partes virtual; Hoja de fiscalización predial</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>8 400 / 340 / 8 900</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Ninguna</t>
+          <t>22 600 predios / pagos del día / 6 200 solicitudes / 1 900</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Rentas y catastro (declarada)</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -574,7 +574,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>500 clientes de la hoja no existen en el ERP; 340 del portal sin vínculo al código del ERP</t>
+          <t>La deuda difiere entre rentas y la hoja de fiscalización</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -589,44 +589,44 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>Maestro de clientes del ERP</t>
+          <t>Padrón de contribuyentes y predios de Rentas y catastro</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>Gerente comercial</t>
+          <t>Subgerente de Administración Tributaria</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Producto</t>
+          <t>Expediente</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>ERP; WMS; Hoja de precios</t>
+          <t>Trámite documentario; Mesa de partes virtual; Hoja de control de expedientes; Archivo físico</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>3 150 / 3 090 / 2 870</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>ERP</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Ninguno</t>
+          <t>6 200 / 6 200 / 6 200 / 6 200 al año</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Ninguna (el físico manda)</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Secretaría General</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>60 SKU sin alta en el WMS; 280 sin precio en la hoja</t>
+          <t>1 340 expedientes sin estado recuperable tras la caída</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -636,210 +636,210 @@
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>Maestro de productos del ERP</t>
+          <t>Expediente electrónico del sistema de gestión documental</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Jefe de compras</t>
+          <t>Secretario General</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Precio</t>
+          <t>Trabajador</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>ERP; Hoja de precios; Portal B2B</t>
+          <t>AIRHSP (MEF); Planilla local; Usuarios de trámite documentario</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>3 150 / 2 870 / 1 200</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Ninguna</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Ninguno</t>
+          <t>178 / 272 con CAS y locación / 124</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>AIRHSP (MEF)</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Recursos Humanos</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>214 precios de la hoja difieren del ERP</t>
+          <t>Los 94 locadores y CAS no figuran en ningún sistema de forma completa</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>Interna</t>
+          <t>Restringida</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí, sensibles</t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>Lista de precios única del ERP</t>
+          <t>AIRHSP para planilla y Planilla local para CAS y locación</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>Gerente comercial</t>
+          <t>Jefe de Recursos Humanos</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Pedido</t>
+          <t>Licencia de funcionamiento</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>ERP; Portal B2B; WMS</t>
+          <t>Trámite documentario; Hoja de registro de licencias; Archivo físico</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>61 200 / 3 670 / 61 050</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>ERP</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>Ninguno</t>
+          <t>410 / 410 / 410 al año</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Ninguna (archivo físico)</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Subgerencia de Licencias</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>150 pedidos del ERP sin orden de preparación en el WMS</t>
+          <t>Plazos distintos en la hoja y en el trámite</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Interna</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Sí (contacto)</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>Registro de pedido del ERP vía capa de integración</t>
+          <t>Registro de licencias del sistema de gestión documental</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Jefe de ventas</t>
+          <t>Subgerente de Licencias</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Comprobante de pago</t>
+          <t>Proveedor</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>ERP; Facturación electrónica</t>
+          <t>SIAF-SP</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>64 800 / 64 800</t>
+          <t>89</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>ERP</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>Contador general</t>
+          <t>SIAF-SP</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Sin discrepancia conocida; contiene contacto y documento de identidad</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Interna</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t>Sí (DNI de personas naturales)</t>
+          <t>Sí (personas naturales)</t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>ERP</t>
+          <t>SIAF-SP</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Contador general</t>
+          <t>Jefe de Logística</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Inventario (stock)</t>
+          <t>Pago a proveedor</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>ERP; WMS</t>
+          <t>SIAF-SP</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>3 150 / 3 090</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Ninguna</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>Jefe de almacén</t>
+          <t>8 126 comprobantes 2025</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>SIAF-SP</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>140 SKU con cantidades distintas al inicio del día</t>
+          <t>Registro y aprobación por usuarios del SIAF sin dueño que responda por el dato</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Interna</t>
+          <t>Confidencial</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -849,29 +849,29 @@
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>Stock del WMS publicado como servicio</t>
+          <t>SIAF-SP</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Jefe de almacén</t>
+          <t>Jefe de Tesorería</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Ruta de despacho</t>
+          <t>Cuenta de usuario</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Hoja de ruteo; WMS (guías)</t>
+          <t>Trámite documentario; Usuarios del ERP (SIAF-SP)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>38 / 38</t>
+          <t>124 / 126</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
@@ -886,183 +886,79 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>Las guías del WMS no reflejan los cambios de ruta del día</t>
+          <t>No se concilian con la planilla (178) ni con el personal CAS y locación (94)</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Restringida</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
-          <t>Sí (conductor)</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>Planificador de rutas integrado al WMS</t>
+          <t>Directorio institucional de cuentas con alta y baja desde Recursos Humanos</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>Jefe de despacho</t>
+          <t>Jefe de la Unidad de TI</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Cuenta por cobrar</t>
+          <t>Acta de registro civil</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>ERP; Hoja de cobranza</t>
+          <t>Libros físicos de registro civil; hojas de cálculo del área</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>2 140 / 2 310</t>
+          <t>Sin conteo: se opera en papel</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Ninguna</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Jefe de créditos y cobranzas</t>
+          <t>Ninguna (papel)</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>170 acuerdos de pago registrados solo en la hoja</t>
+          <t>No existe índice digital de las actas</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Confidencial</t>
+          <t>Restringida</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Sí, sensibles</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>ERP (módulo Créditos)</t>
+          <t>Sistema de registro civil integrado con RENIEC</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Jefe de créditos y cobranzas</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Trabajador</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Planilla; ERP; Hoja de personal</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>48 / 52 / 48</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Planilla</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Jefe de RR. HH.</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>4 usuarios del ERP pertenecen a personal cesado</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>Restringida</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>Sí, sensibles</t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>Sistema de planilla</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>Jefe de RR. HH.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Proveedor</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>ERP</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>410</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>ERP</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>Jefe de compras</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr">
-        <is>
-          <t>Interna</t>
-        </is>
-      </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>ERP</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>Jefe de compras</t>
+          <t>Jefe de Registro Civil</t>
         </is>
       </c>
     </row>
@@ -1077,7 +973,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1098,7 +994,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>DICOSUR · PETI v0.10 · Restringido · Taller 10 SI-886</t>
+          <t>Municipalidad Distrital de Alto Selva · PETI v0.10 · Restringido · Taller 10 SI-886</t>
         </is>
       </c>
     </row>
@@ -1142,27 +1038,27 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Abastecimiento</t>
+          <t>Trámite documentario y mesa de partes</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>ERP Compras</t>
+          <t>Trámite documentario (sin soporte) + hoja de expedientes</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>APP-01</t>
+          <t>APP-02; APP-06</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Bueno</t>
+          <t>Deficiente</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Órdenes de compra y recepción registradas en el ERP</t>
+          <t>Sin documentación ni soporte; el físico manda; 1 340 expedientes sin estado tras la caída</t>
         </is>
       </c>
     </row>
@@ -1174,27 +1070,27 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Toma de pedido</t>
+          <t>Recaudación de tributos municipales</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Teléfono + papel + Portal B2B (6 %)</t>
+          <t>Rentas y catastro (sin soporte) + hoja de fiscalización</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>APP-02; APP-08</t>
+          <t>APP-03; APP-07</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Deficiente</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>94 % de los pedidos por teléfono o papel; los del portal se vuelven a digitar (INT-02)</t>
+          <t>Sistema operativo pero sin soporte; caído 9 días hábiles en 2025; se digita al SIAF-SP al cierre</t>
         </is>
       </c>
     </row>
@@ -1206,27 +1102,27 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Aprobación de crédito</t>
+          <t>Licencias de funcionamiento y edificación</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>ERP Créditos</t>
+          <t>Rentas y catastro + HOJA DE LICENCIAS + archivo físico</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>APP-01</t>
+          <t>APP-03; APP-08</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Bueno</t>
+          <t>Deficiente</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>Límite de crédito por cliente controlado en el ERP</t>
+          <t>La fuente es el archivo físico; plazos distintos en la hoja y en el trámite</t>
         </is>
       </c>
     </row>
@@ -1238,27 +1134,27 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Preparación del pedido</t>
+          <t>Registro civil</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>WMS + lectores de código de barras</t>
+          <t>NINGUNO · papel y hojas de cálculo</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>APP-03</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Bueno</t>
+          <t>Sin soporte</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Preparación con lectura de código; stock sincronizado de noche (INT-01)</t>
+          <t>Actas solo en libros físicos; sin índice digital</t>
         </is>
       </c>
     </row>
@@ -1270,27 +1166,27 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Ruteo y despacho</t>
+          <t>Contrataciones y logística</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>HOJA DE CÁLCULO de ruteo</t>
+          <t>SIAF-SP (MEF)</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>APP-06</t>
+          <t>APP-01</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Deficiente</t>
+          <t>Bueno</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>38 rutas armadas a mano cada noche; 22 % del costo operativo</t>
+          <t>Sistema obligatorio con soporte del MEF</t>
         </is>
       </c>
     </row>
@@ -1302,27 +1198,27 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Facturación</t>
+          <t>Atención al ciudadano</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>ERP Ventas + facturación electrónica</t>
+          <t>Mesa de partes virtual (formulario + correo)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>APP-01; APP-05</t>
+          <t>APP-05</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Bueno</t>
+          <t>Deficiente</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Comprobantes emitidos en línea (INT-04)</t>
+          <t>El correo se imprime y se vuelve a registrar; sin soporte</t>
         </is>
       </c>
     </row>
@@ -1334,17 +1230,17 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Cobranza</t>
+          <t>Gestión de personal y planilla</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>ERP + hoja de cálculo de cobranza</t>
+          <t>AIRHSP (MEF) + Planilla local</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>APP-01; APP-09</t>
+          <t>APP-09; APP-10</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1354,7 +1250,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>170 acuerdos de pago existen solo en la hoja</t>
+          <t>Los locadores no figuran en ningún sistema</t>
         </is>
       </c>
     </row>
@@ -1366,91 +1262,27 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Atención de reclamos</t>
+          <t>Transparencia y acceso a la información</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>CORREO electrónico</t>
+          <t>Portal de transparencia estándar (PCM)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>APP-12</t>
+          <t>APP-04</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Deficiente</t>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Sin registro ni seguimiento del reclamo</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>PRO-09</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Análisis comercial y reportes</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>HOJAS DE CÁLCULO</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>APP-07; APP-11</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Deficiente</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>Reportes armados a mano en 3 días al cierre de cada mes</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>PRO-10</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Gestión de personal y planilla</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Sistema de planilla + hoja de personal</t>
-        </is>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>APP-04; APP-10</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>Parcial</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Planilla en sistema; datos de personal duplicados en hoja</t>
+          <t>La plataforma tiene soporte de la PCM pero se carga a mano</t>
         </is>
       </c>
     </row>
@@ -1509,11 +1341,11 @@
         </is>
       </c>
       <c r="B5" s="7">
-        <f>COUNTIF(Entidades!D5:D14,"Ninguna")</f>
+        <f>COUNTIF(Entidades!D5:D12,"Ninguna*")</f>
         <v/>
       </c>
       <c r="C5" s="7">
-        <f>COUNTA(Entidades!A5:A14)</f>
+        <f>COUNTA(Entidades!A5:A12)</f>
         <v/>
       </c>
     </row>
@@ -1524,11 +1356,11 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>COUNTIF(Entidades!E5:E14,"Ninguno")</f>
+        <f>COUNTIF(Entidades!E5:E12,"Ninguno")</f>
         <v/>
       </c>
       <c r="C6" s="7">
-        <f>COUNTA(Entidades!A5:A14)</f>
+        <f>COUNTA(Entidades!A5:A12)</f>
         <v/>
       </c>
     </row>
@@ -1539,11 +1371,11 @@
         </is>
       </c>
       <c r="B7" s="7">
-        <f>COUNTIFS(Entidades!D5:D14,"Ninguna",Entidades!E5:E14,"Ninguno")</f>
+        <f>COUNTIFS(Entidades!D5:D12,"Ninguna*",Entidades!E5:E12,"Ninguno")</f>
         <v/>
       </c>
       <c r="C7" s="7">
-        <f>COUNTA(Entidades!A5:A14)</f>
+        <f>COUNTA(Entidades!A5:A12)</f>
         <v/>
       </c>
     </row>
@@ -1554,26 +1386,26 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>COUNTIF(Entidades!H5:H14,"Sí*")</f>
+        <f>COUNTIF(Entidades!H5:H12,"Sí*")</f>
         <v/>
       </c>
       <c r="C8" s="7">
-        <f>COUNTA(Entidades!A5:A14)</f>
+        <f>COUNTA(Entidades!A5:A12)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Procesos con soporte deficiente</t>
+          <t>Procesos sin soporte o con soporte deficiente</t>
         </is>
       </c>
       <c r="B9" s="7">
-        <f>COUNTIF(Cooperación!E5:E14,"Deficiente")</f>
+        <f>COUNTIF(Cooperación!E5:E12,"Deficiente")+COUNTIF(Cooperación!E5:E12,"Sin soporte")</f>
         <v/>
       </c>
       <c r="C9" s="7">
-        <f>COUNTA(Cooperación!A5:A14)</f>
+        <f>COUNTA(Cooperación!A5:A12)</f>
         <v/>
       </c>
     </row>
@@ -1584,11 +1416,11 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>COUNTIF(Cooperación!E5:E14,"Parcial")</f>
+        <f>COUNTIF(Cooperación!E5:E12,"Parcial")</f>
         <v/>
       </c>
       <c r="C10" s="7">
-        <f>COUNTA(Cooperación!A5:A14)</f>
+        <f>COUNTA(Cooperación!A5:A12)</f>
         <v/>
       </c>
     </row>

</xml_diff>